<commit_message>
Add Portfolio roll-up tab to valuation template
Standalone tab with one row per property (dropdowns for type and tenanted).
Each row auto-computes passing rent, NOI, net yield, income value, comparable
value, indicative value, and gain. Totals row plus KPI callouts roll up total
invested, total value, total gain, total return, and blended net yield across
the whole portfolio.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01F34pBmQnkApCzfs23gFMM6
</commit_message>
<xml_diff>
--- a/Property_Valuation_Template.xlsx
+++ b/Property_Valuation_Template.xlsx
@@ -8,12 +8,13 @@
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Inputs" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Income Schedule" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Valuation" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="DCF" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Net Proceeds" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Returns" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Portfolio" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Inputs" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Income Schedule" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Valuation" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="DCF" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Net Proceeds" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Returns" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Summary'!$A$1:$D$20</definedName>
@@ -24,15 +25,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="6">
+  <numFmts count="7">
     <numFmt numFmtId="164" formatCode="#,##0 &quot;AED&quot;"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="#,##0 &quot;AED/sqft&quot;"/>
     <numFmt numFmtId="167" formatCode="+#,##0 &quot;AED&quot;;-#,##0 &quot;AED&quot;"/>
     <numFmt numFmtId="168" formatCode="0.000"/>
     <numFmt numFmtId="169" formatCode="0.0"/>
+    <numFmt numFmtId="170" formatCode="+#,##0;-#,##0"/>
   </numFmts>
-  <fonts count="19">
+  <fonts count="23">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -121,8 +123,26 @@
     <font>
       <sz val="10"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F3864"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="13"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -164,6 +184,11 @@
         <fgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00548235"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="3">
     <border>
@@ -192,7 +217,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="86">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="15" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -345,6 +370,79 @@
     </xf>
     <xf numFmtId="165" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="20" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="20" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="20" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="20" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="22" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="22" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="22" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="22" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -929,6 +1027,811 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:S22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="7" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="9" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="8" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
+    <col width="15" customWidth="1" min="18" max="18"/>
+    <col width="15" customWidth="1" min="19" max="19"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="13" t="inlineStr">
+        <is>
+          <t>PORTFOLIO ROLL-UP  —  one row per property</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="24" customHeight="1">
+      <c r="A2" s="61" t="inlineStr">
+        <is>
+          <t>Standalone tab (does NOT depend on the Inputs tab). Fill the GOLD input columns for each property; values &amp; totals auto-calculate. Tenanted → income value; Vacant → comparable (area × psf).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="62" t="inlineStr">
+        <is>
+          <t>INPUTS  (edit these)</t>
+        </is>
+      </c>
+      <c r="M3" s="63" t="inlineStr">
+        <is>
+          <t>AUTO-CALCULATED</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="64" t="inlineStr">
+        <is>
+          <t>Property</t>
+        </is>
+      </c>
+      <c r="B4" s="64" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C4" s="64" t="inlineStr">
+        <is>
+          <t>Tenanted?</t>
+        </is>
+      </c>
+      <c r="D4" s="64" t="inlineStr">
+        <is>
+          <t>Area sqft</t>
+        </is>
+      </c>
+      <c r="E4" s="64" t="inlineStr">
+        <is>
+          <t>Cost (AED)</t>
+        </is>
+      </c>
+      <c r="F4" s="64" t="inlineStr">
+        <is>
+          <t>Yr-1 Rent</t>
+        </is>
+      </c>
+      <c r="G4" s="64" t="inlineStr">
+        <is>
+          <t>Esc %</t>
+        </is>
+      </c>
+      <c r="H4" s="64" t="inlineStr">
+        <is>
+          <t>Cur Yr</t>
+        </is>
+      </c>
+      <c r="I4" s="64" t="inlineStr">
+        <is>
+          <t>Term</t>
+        </is>
+      </c>
+      <c r="J4" s="64" t="inlineStr">
+        <is>
+          <t>Ann. Service Chg</t>
+        </is>
+      </c>
+      <c r="K4" s="64" t="inlineStr">
+        <is>
+          <t>AED/sqft</t>
+        </is>
+      </c>
+      <c r="L4" s="64" t="inlineStr">
+        <is>
+          <t>Target Yld</t>
+        </is>
+      </c>
+      <c r="M4" s="65" t="inlineStr">
+        <is>
+          <t>Passing Rent</t>
+        </is>
+      </c>
+      <c r="N4" s="65" t="inlineStr">
+        <is>
+          <t>NOI</t>
+        </is>
+      </c>
+      <c r="O4" s="65" t="inlineStr">
+        <is>
+          <t>Net Yld</t>
+        </is>
+      </c>
+      <c r="P4" s="65" t="inlineStr">
+        <is>
+          <t>Income Value</t>
+        </is>
+      </c>
+      <c r="Q4" s="65" t="inlineStr">
+        <is>
+          <t>Comparable</t>
+        </is>
+      </c>
+      <c r="R4" s="65" t="inlineStr">
+        <is>
+          <t>Indicative Value</t>
+        </is>
+      </c>
+      <c r="S4" s="65" t="inlineStr">
+        <is>
+          <t>Gain vs Cost</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="66" t="inlineStr">
+        <is>
+          <t>Office – Business Bay</t>
+        </is>
+      </c>
+      <c r="B5" s="66" t="inlineStr">
+        <is>
+          <t>Office</t>
+        </is>
+      </c>
+      <c r="C5" s="66" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D5" s="18" t="n">
+        <v>1200</v>
+      </c>
+      <c r="E5" s="19" t="n">
+        <v>4550000</v>
+      </c>
+      <c r="F5" s="19" t="n">
+        <v>465992</v>
+      </c>
+      <c r="G5" s="67" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="H5" s="68" t="n">
+        <v>2</v>
+      </c>
+      <c r="I5" s="68" t="n">
+        <v>5</v>
+      </c>
+      <c r="J5" s="19" t="n">
+        <v>40000</v>
+      </c>
+      <c r="K5" s="18" t="n">
+        <v>4200</v>
+      </c>
+      <c r="L5" s="67" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="M5" s="28">
+        <f>IF(C5="Yes",F5*(1+G5)^(H5-1),0)</f>
+        <v/>
+      </c>
+      <c r="N5" s="28">
+        <f>IF(M5=0,0,M5-J5)</f>
+        <v/>
+      </c>
+      <c r="O5" s="69">
+        <f>IF(E5&gt;0,N5/E5,0)</f>
+        <v/>
+      </c>
+      <c r="P5" s="28">
+        <f>IF(M5=0,"",N5/L5)</f>
+        <v/>
+      </c>
+      <c r="Q5" s="28">
+        <f>IF(N(D5)*N(K5)=0,"",D5*K5)</f>
+        <v/>
+      </c>
+      <c r="R5" s="51">
+        <f>IF(M5&gt;0,N5/L5,IF(N(D5)*N(K5)=0,0,D5*K5))</f>
+        <v/>
+      </c>
+      <c r="S5" s="70">
+        <f>IF(R5=0,"",R5-E5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="66" t="n"/>
+      <c r="B6" s="66" t="n"/>
+      <c r="C6" s="66" t="n"/>
+      <c r="D6" s="18" t="n"/>
+      <c r="E6" s="19" t="n"/>
+      <c r="F6" s="19" t="n"/>
+      <c r="G6" s="67" t="n"/>
+      <c r="H6" s="68" t="n"/>
+      <c r="I6" s="68" t="n"/>
+      <c r="J6" s="19" t="n"/>
+      <c r="K6" s="18" t="n"/>
+      <c r="L6" s="67" t="n"/>
+      <c r="M6" s="31">
+        <f>IF(C6="Yes",F6*(1+G6)^(H6-1),0)</f>
+        <v/>
+      </c>
+      <c r="N6" s="31">
+        <f>IF(M6=0,0,M6-J6)</f>
+        <v/>
+      </c>
+      <c r="O6" s="71">
+        <f>IF(E6&gt;0,N6/E6,0)</f>
+        <v/>
+      </c>
+      <c r="P6" s="31">
+        <f>IF(M6=0,"",N6/L6)</f>
+        <v/>
+      </c>
+      <c r="Q6" s="31">
+        <f>IF(N(D6)*N(K6)=0,"",D6*K6)</f>
+        <v/>
+      </c>
+      <c r="R6" s="54">
+        <f>IF(M6&gt;0,N6/L6,IF(N(D6)*N(K6)=0,0,D6*K6))</f>
+        <v/>
+      </c>
+      <c r="S6" s="72">
+        <f>IF(R6=0,"",R6-E6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="66" t="n"/>
+      <c r="B7" s="66" t="n"/>
+      <c r="C7" s="66" t="n"/>
+      <c r="D7" s="18" t="n"/>
+      <c r="E7" s="19" t="n"/>
+      <c r="F7" s="19" t="n"/>
+      <c r="G7" s="67" t="n"/>
+      <c r="H7" s="68" t="n"/>
+      <c r="I7" s="68" t="n"/>
+      <c r="J7" s="19" t="n"/>
+      <c r="K7" s="18" t="n"/>
+      <c r="L7" s="67" t="n"/>
+      <c r="M7" s="28">
+        <f>IF(C7="Yes",F7*(1+G7)^(H7-1),0)</f>
+        <v/>
+      </c>
+      <c r="N7" s="28">
+        <f>IF(M7=0,0,M7-J7)</f>
+        <v/>
+      </c>
+      <c r="O7" s="69">
+        <f>IF(E7&gt;0,N7/E7,0)</f>
+        <v/>
+      </c>
+      <c r="P7" s="28">
+        <f>IF(M7=0,"",N7/L7)</f>
+        <v/>
+      </c>
+      <c r="Q7" s="28">
+        <f>IF(N(D7)*N(K7)=0,"",D7*K7)</f>
+        <v/>
+      </c>
+      <c r="R7" s="51">
+        <f>IF(M7&gt;0,N7/L7,IF(N(D7)*N(K7)=0,0,D7*K7))</f>
+        <v/>
+      </c>
+      <c r="S7" s="70">
+        <f>IF(R7=0,"",R7-E7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="66" t="n"/>
+      <c r="B8" s="66" t="n"/>
+      <c r="C8" s="66" t="n"/>
+      <c r="D8" s="18" t="n"/>
+      <c r="E8" s="19" t="n"/>
+      <c r="F8" s="19" t="n"/>
+      <c r="G8" s="67" t="n"/>
+      <c r="H8" s="68" t="n"/>
+      <c r="I8" s="68" t="n"/>
+      <c r="J8" s="19" t="n"/>
+      <c r="K8" s="18" t="n"/>
+      <c r="L8" s="67" t="n"/>
+      <c r="M8" s="31">
+        <f>IF(C8="Yes",F8*(1+G8)^(H8-1),0)</f>
+        <v/>
+      </c>
+      <c r="N8" s="31">
+        <f>IF(M8=0,0,M8-J8)</f>
+        <v/>
+      </c>
+      <c r="O8" s="71">
+        <f>IF(E8&gt;0,N8/E8,0)</f>
+        <v/>
+      </c>
+      <c r="P8" s="31">
+        <f>IF(M8=0,"",N8/L8)</f>
+        <v/>
+      </c>
+      <c r="Q8" s="31">
+        <f>IF(N(D8)*N(K8)=0,"",D8*K8)</f>
+        <v/>
+      </c>
+      <c r="R8" s="54">
+        <f>IF(M8&gt;0,N8/L8,IF(N(D8)*N(K8)=0,0,D8*K8))</f>
+        <v/>
+      </c>
+      <c r="S8" s="72">
+        <f>IF(R8=0,"",R8-E8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="66" t="n"/>
+      <c r="B9" s="66" t="n"/>
+      <c r="C9" s="66" t="n"/>
+      <c r="D9" s="18" t="n"/>
+      <c r="E9" s="19" t="n"/>
+      <c r="F9" s="19" t="n"/>
+      <c r="G9" s="67" t="n"/>
+      <c r="H9" s="68" t="n"/>
+      <c r="I9" s="68" t="n"/>
+      <c r="J9" s="19" t="n"/>
+      <c r="K9" s="18" t="n"/>
+      <c r="L9" s="67" t="n"/>
+      <c r="M9" s="28">
+        <f>IF(C9="Yes",F9*(1+G9)^(H9-1),0)</f>
+        <v/>
+      </c>
+      <c r="N9" s="28">
+        <f>IF(M9=0,0,M9-J9)</f>
+        <v/>
+      </c>
+      <c r="O9" s="69">
+        <f>IF(E9&gt;0,N9/E9,0)</f>
+        <v/>
+      </c>
+      <c r="P9" s="28">
+        <f>IF(M9=0,"",N9/L9)</f>
+        <v/>
+      </c>
+      <c r="Q9" s="28">
+        <f>IF(N(D9)*N(K9)=0,"",D9*K9)</f>
+        <v/>
+      </c>
+      <c r="R9" s="51">
+        <f>IF(M9&gt;0,N9/L9,IF(N(D9)*N(K9)=0,0,D9*K9))</f>
+        <v/>
+      </c>
+      <c r="S9" s="70">
+        <f>IF(R9=0,"",R9-E9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="66" t="n"/>
+      <c r="B10" s="66" t="n"/>
+      <c r="C10" s="66" t="n"/>
+      <c r="D10" s="18" t="n"/>
+      <c r="E10" s="19" t="n"/>
+      <c r="F10" s="19" t="n"/>
+      <c r="G10" s="67" t="n"/>
+      <c r="H10" s="68" t="n"/>
+      <c r="I10" s="68" t="n"/>
+      <c r="J10" s="19" t="n"/>
+      <c r="K10" s="18" t="n"/>
+      <c r="L10" s="67" t="n"/>
+      <c r="M10" s="31">
+        <f>IF(C10="Yes",F10*(1+G10)^(H10-1),0)</f>
+        <v/>
+      </c>
+      <c r="N10" s="31">
+        <f>IF(M10=0,0,M10-J10)</f>
+        <v/>
+      </c>
+      <c r="O10" s="71">
+        <f>IF(E10&gt;0,N10/E10,0)</f>
+        <v/>
+      </c>
+      <c r="P10" s="31">
+        <f>IF(M10=0,"",N10/L10)</f>
+        <v/>
+      </c>
+      <c r="Q10" s="31">
+        <f>IF(N(D10)*N(K10)=0,"",D10*K10)</f>
+        <v/>
+      </c>
+      <c r="R10" s="54">
+        <f>IF(M10&gt;0,N10/L10,IF(N(D10)*N(K10)=0,0,D10*K10))</f>
+        <v/>
+      </c>
+      <c r="S10" s="72">
+        <f>IF(R10=0,"",R10-E10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="66" t="n"/>
+      <c r="B11" s="66" t="n"/>
+      <c r="C11" s="66" t="n"/>
+      <c r="D11" s="18" t="n"/>
+      <c r="E11" s="19" t="n"/>
+      <c r="F11" s="19" t="n"/>
+      <c r="G11" s="67" t="n"/>
+      <c r="H11" s="68" t="n"/>
+      <c r="I11" s="68" t="n"/>
+      <c r="J11" s="19" t="n"/>
+      <c r="K11" s="18" t="n"/>
+      <c r="L11" s="67" t="n"/>
+      <c r="M11" s="28">
+        <f>IF(C11="Yes",F11*(1+G11)^(H11-1),0)</f>
+        <v/>
+      </c>
+      <c r="N11" s="28">
+        <f>IF(M11=0,0,M11-J11)</f>
+        <v/>
+      </c>
+      <c r="O11" s="69">
+        <f>IF(E11&gt;0,N11/E11,0)</f>
+        <v/>
+      </c>
+      <c r="P11" s="28">
+        <f>IF(M11=0,"",N11/L11)</f>
+        <v/>
+      </c>
+      <c r="Q11" s="28">
+        <f>IF(N(D11)*N(K11)=0,"",D11*K11)</f>
+        <v/>
+      </c>
+      <c r="R11" s="51">
+        <f>IF(M11&gt;0,N11/L11,IF(N(D11)*N(K11)=0,0,D11*K11))</f>
+        <v/>
+      </c>
+      <c r="S11" s="70">
+        <f>IF(R11=0,"",R11-E11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="66" t="n"/>
+      <c r="B12" s="66" t="n"/>
+      <c r="C12" s="66" t="n"/>
+      <c r="D12" s="18" t="n"/>
+      <c r="E12" s="19" t="n"/>
+      <c r="F12" s="19" t="n"/>
+      <c r="G12" s="67" t="n"/>
+      <c r="H12" s="68" t="n"/>
+      <c r="I12" s="68" t="n"/>
+      <c r="J12" s="19" t="n"/>
+      <c r="K12" s="18" t="n"/>
+      <c r="L12" s="67" t="n"/>
+      <c r="M12" s="31">
+        <f>IF(C12="Yes",F12*(1+G12)^(H12-1),0)</f>
+        <v/>
+      </c>
+      <c r="N12" s="31">
+        <f>IF(M12=0,0,M12-J12)</f>
+        <v/>
+      </c>
+      <c r="O12" s="71">
+        <f>IF(E12&gt;0,N12/E12,0)</f>
+        <v/>
+      </c>
+      <c r="P12" s="31">
+        <f>IF(M12=0,"",N12/L12)</f>
+        <v/>
+      </c>
+      <c r="Q12" s="31">
+        <f>IF(N(D12)*N(K12)=0,"",D12*K12)</f>
+        <v/>
+      </c>
+      <c r="R12" s="54">
+        <f>IF(M12&gt;0,N12/L12,IF(N(D12)*N(K12)=0,0,D12*K12))</f>
+        <v/>
+      </c>
+      <c r="S12" s="72">
+        <f>IF(R12=0,"",R12-E12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="66" t="n"/>
+      <c r="B13" s="66" t="n"/>
+      <c r="C13" s="66" t="n"/>
+      <c r="D13" s="18" t="n"/>
+      <c r="E13" s="19" t="n"/>
+      <c r="F13" s="19" t="n"/>
+      <c r="G13" s="67" t="n"/>
+      <c r="H13" s="68" t="n"/>
+      <c r="I13" s="68" t="n"/>
+      <c r="J13" s="19" t="n"/>
+      <c r="K13" s="18" t="n"/>
+      <c r="L13" s="67" t="n"/>
+      <c r="M13" s="28">
+        <f>IF(C13="Yes",F13*(1+G13)^(H13-1),0)</f>
+        <v/>
+      </c>
+      <c r="N13" s="28">
+        <f>IF(M13=0,0,M13-J13)</f>
+        <v/>
+      </c>
+      <c r="O13" s="69">
+        <f>IF(E13&gt;0,N13/E13,0)</f>
+        <v/>
+      </c>
+      <c r="P13" s="28">
+        <f>IF(M13=0,"",N13/L13)</f>
+        <v/>
+      </c>
+      <c r="Q13" s="28">
+        <f>IF(N(D13)*N(K13)=0,"",D13*K13)</f>
+        <v/>
+      </c>
+      <c r="R13" s="51">
+        <f>IF(M13&gt;0,N13/L13,IF(N(D13)*N(K13)=0,0,D13*K13))</f>
+        <v/>
+      </c>
+      <c r="S13" s="70">
+        <f>IF(R13=0,"",R13-E13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="66" t="n"/>
+      <c r="B14" s="66" t="n"/>
+      <c r="C14" s="66" t="n"/>
+      <c r="D14" s="18" t="n"/>
+      <c r="E14" s="19" t="n"/>
+      <c r="F14" s="19" t="n"/>
+      <c r="G14" s="67" t="n"/>
+      <c r="H14" s="68" t="n"/>
+      <c r="I14" s="68" t="n"/>
+      <c r="J14" s="19" t="n"/>
+      <c r="K14" s="18" t="n"/>
+      <c r="L14" s="67" t="n"/>
+      <c r="M14" s="31">
+        <f>IF(C14="Yes",F14*(1+G14)^(H14-1),0)</f>
+        <v/>
+      </c>
+      <c r="N14" s="31">
+        <f>IF(M14=0,0,M14-J14)</f>
+        <v/>
+      </c>
+      <c r="O14" s="71">
+        <f>IF(E14&gt;0,N14/E14,0)</f>
+        <v/>
+      </c>
+      <c r="P14" s="31">
+        <f>IF(M14=0,"",N14/L14)</f>
+        <v/>
+      </c>
+      <c r="Q14" s="31">
+        <f>IF(N(D14)*N(K14)=0,"",D14*K14)</f>
+        <v/>
+      </c>
+      <c r="R14" s="54">
+        <f>IF(M14&gt;0,N14/L14,IF(N(D14)*N(K14)=0,0,D14*K14))</f>
+        <v/>
+      </c>
+      <c r="S14" s="72">
+        <f>IF(R14=0,"",R14-E14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="66" t="n"/>
+      <c r="B15" s="66" t="n"/>
+      <c r="C15" s="66" t="n"/>
+      <c r="D15" s="18" t="n"/>
+      <c r="E15" s="19" t="n"/>
+      <c r="F15" s="19" t="n"/>
+      <c r="G15" s="67" t="n"/>
+      <c r="H15" s="68" t="n"/>
+      <c r="I15" s="68" t="n"/>
+      <c r="J15" s="19" t="n"/>
+      <c r="K15" s="18" t="n"/>
+      <c r="L15" s="67" t="n"/>
+      <c r="M15" s="28">
+        <f>IF(C15="Yes",F15*(1+G15)^(H15-1),0)</f>
+        <v/>
+      </c>
+      <c r="N15" s="28">
+        <f>IF(M15=0,0,M15-J15)</f>
+        <v/>
+      </c>
+      <c r="O15" s="69">
+        <f>IF(E15&gt;0,N15/E15,0)</f>
+        <v/>
+      </c>
+      <c r="P15" s="28">
+        <f>IF(M15=0,"",N15/L15)</f>
+        <v/>
+      </c>
+      <c r="Q15" s="28">
+        <f>IF(N(D15)*N(K15)=0,"",D15*K15)</f>
+        <v/>
+      </c>
+      <c r="R15" s="51">
+        <f>IF(M15&gt;0,N15/L15,IF(N(D15)*N(K15)=0,0,D15*K15))</f>
+        <v/>
+      </c>
+      <c r="S15" s="70">
+        <f>IF(R15=0,"",R15-E15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="66" t="n"/>
+      <c r="B16" s="66" t="n"/>
+      <c r="C16" s="66" t="n"/>
+      <c r="D16" s="18" t="n"/>
+      <c r="E16" s="19" t="n"/>
+      <c r="F16" s="19" t="n"/>
+      <c r="G16" s="67" t="n"/>
+      <c r="H16" s="68" t="n"/>
+      <c r="I16" s="68" t="n"/>
+      <c r="J16" s="19" t="n"/>
+      <c r="K16" s="18" t="n"/>
+      <c r="L16" s="67" t="n"/>
+      <c r="M16" s="31">
+        <f>IF(C16="Yes",F16*(1+G16)^(H16-1),0)</f>
+        <v/>
+      </c>
+      <c r="N16" s="31">
+        <f>IF(M16=0,0,M16-J16)</f>
+        <v/>
+      </c>
+      <c r="O16" s="71">
+        <f>IF(E16&gt;0,N16/E16,0)</f>
+        <v/>
+      </c>
+      <c r="P16" s="31">
+        <f>IF(M16=0,"",N16/L16)</f>
+        <v/>
+      </c>
+      <c r="Q16" s="31">
+        <f>IF(N(D16)*N(K16)=0,"",D16*K16)</f>
+        <v/>
+      </c>
+      <c r="R16" s="54">
+        <f>IF(M16&gt;0,N16/L16,IF(N(D16)*N(K16)=0,0,D16*K16))</f>
+        <v/>
+      </c>
+      <c r="S16" s="72">
+        <f>IF(R16=0,"",R16-E16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="73" t="inlineStr">
+        <is>
+          <t>PORTFOLIO TOTAL</t>
+        </is>
+      </c>
+      <c r="B17" s="74" t="n"/>
+      <c r="C17" s="74" t="n"/>
+      <c r="D17" s="75">
+        <f>SUM(D5:D16)</f>
+        <v/>
+      </c>
+      <c r="E17" s="76">
+        <f>SUM(E5:E16)</f>
+        <v/>
+      </c>
+      <c r="F17" s="77" t="n"/>
+      <c r="G17" s="77" t="n"/>
+      <c r="H17" s="77" t="n"/>
+      <c r="I17" s="77" t="n"/>
+      <c r="J17" s="77" t="n"/>
+      <c r="K17" s="77" t="n"/>
+      <c r="L17" s="77" t="n"/>
+      <c r="M17" s="77" t="n"/>
+      <c r="N17" s="76">
+        <f>SUM(N5:N16)</f>
+        <v/>
+      </c>
+      <c r="O17" s="78">
+        <f>IF(SUM(E5:E16)&gt;0,SUM(N5:N16)/SUM(E5:E16),0)</f>
+        <v/>
+      </c>
+      <c r="P17" s="77" t="n"/>
+      <c r="Q17" s="77" t="n"/>
+      <c r="R17" s="76">
+        <f>SUM(R5:R16)</f>
+        <v/>
+      </c>
+      <c r="S17" s="79">
+        <f>SUM(S5:S16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="80" t="inlineStr">
+        <is>
+          <t>Total invested</t>
+        </is>
+      </c>
+      <c r="C19" s="80" t="inlineStr">
+        <is>
+          <t>Total value</t>
+        </is>
+      </c>
+      <c r="E19" s="80" t="inlineStr">
+        <is>
+          <t>Total gain</t>
+        </is>
+      </c>
+      <c r="G19" s="80" t="inlineStr">
+        <is>
+          <t>Total return</t>
+        </is>
+      </c>
+      <c r="I19" s="80" t="inlineStr">
+        <is>
+          <t>Blended net yield</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="81">
+        <f>E17</f>
+        <v/>
+      </c>
+      <c r="C20" s="82">
+        <f>R17</f>
+        <v/>
+      </c>
+      <c r="E20" s="83">
+        <f>S17</f>
+        <v/>
+      </c>
+      <c r="G20" s="84">
+        <f>IF(E17&gt;0,S17/E17,0)</f>
+        <v/>
+      </c>
+      <c r="I20" s="85">
+        <f>O17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="12" t="inlineStr">
+        <is>
+          <t>Blended net yield = total NOI ÷ total invested. 'Indicative' uses income value for tenanted units, comparable (area × AED/sqft) for vacant. Gain ignores selling costs.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A3:L3"/>
+    <mergeCell ref="A2:S2"/>
+    <mergeCell ref="M3:S3"/>
+    <mergeCell ref="A1:S1"/>
+  </mergeCells>
+  <dataValidations count="2">
+    <dataValidation sqref="B5:B16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Apartment,Villa,Townhouse,Office,Retail,Warehouse,Land/Plot,Off-plan,Other"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C5:C16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1362,7 +2265,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1584,7 +2487,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1802,7 +2705,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2144,7 +3047,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2343,7 +3246,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>